<commit_message>
Accreditamento FSE: aggiunta documentazione di test Fix report-checklist.xlsx [48,475]
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#VASHLABSSNCXX/VASHLABS/TELERICETTA/2.0.21/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/A1#111#VASHLABSSNCXX/VASHLABS/TELERICETTA/2.0.21/accreditamento-checklist_V8.3.0.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\00_TELERICETTA\01_SVILUPPO\04_SDK_SOGEI\13_FSE\00_REPO_GIT_ACCREDITAMENTO\00_SRV_SEBA_repository_20260316\repository\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NetBeansProgettiSviluppo\06_FSE_ACCREDITAMENTO_GIT\it-fse-accreditamento\GATEWAY\A1#111#VASHLABSSNCXX\VASHLABS\TELERICETTA\2.0.21\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E993C109-C444-4C8D-9916-9DDCED25F359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08B57CE0-222E-4101-BA3E-DC759EAA74D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1398" uniqueCount="571">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -5313,7 +5313,9 @@
       <c r="G31" s="35"/>
       <c r="H31" s="35"/>
       <c r="I31" s="40"/>
-      <c r="J31" s="36"/>
+      <c r="J31" s="36" t="s">
+        <v>76</v>
+      </c>
       <c r="L31" s="36"/>
       <c r="M31" s="36" t="s">
         <v>76</v>
@@ -11355,7 +11357,9 @@
       <c r="I190" s="40" t="s">
         <v>557</v>
       </c>
-      <c r="J190" s="36"/>
+      <c r="J190" s="36" t="s">
+        <v>76</v>
+      </c>
       <c r="K190" s="36"/>
       <c r="L190" s="36"/>
       <c r="M190" s="36" t="s">
@@ -18732,27 +18736,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -19016,32 +18999,28 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19060,6 +19039,31 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>

<commit_message>
Accreditamento FSE: aggiunta documentazione di test Fix dati dopo review 17/03/2026 17:19
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#VASHLABSSNCXX/VASHLABS/TELERICETTA/2.0.21/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/A1#111#VASHLABSSNCXX/VASHLABS/TELERICETTA/2.0.21/accreditamento-checklist_V8.3.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NetBeansProgettiSviluppo\06_FSE_ACCREDITAMENTO_GIT\it-fse-accreditamento\GATEWAY\A1#111#VASHLABSSNCXX\VASHLABS\TELERICETTA\2.0.21\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08B57CE0-222E-4101-BA3E-DC759EAA74D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9145B25C-7895-4313-B51E-EC5E31D964B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2092,60 +2092,15 @@
     <t>La richiesta di validazione fallisce in modo sincrono, viene restituito errore al chiamante, l’evento viene tracciato nei log/backoffice, non viene accodata alcuna ritrasmissione automatica; dopo la risoluzione del problema il documento deve essere reinviato manualmente dal sistema chiamante.</t>
   </si>
   <si>
-    <t>eaa4b513aa25c46ded83347d9e8d72cb</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.cb9c6b3773^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.6.103, Codes: INVALID-CODE, 88.35.1]</t>
   </si>
   <si>
-    <t>17:20:56+00:00</t>
-  </si>
-  <si>
-    <t>16:54:30+00:00</t>
-  </si>
-  <si>
-    <t>c158cdbf5a584901d32625926aec00ec</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.98289dd2d4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.6.103, Codes: INVALID-RELATIVE-CODE, 88.35.1]</t>
   </si>
   <si>
-    <t>e61d1f0943613e5173cf4ce13191486f</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.110b06b86e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.5.7 v2.1.0, Codes: NOT-VALID], [CodeSystem: 2.16.840.1.113883.6.103, Codes: 88.35.1]</t>
   </si>
   <si>
-    <t>17:34:43+00:00</t>
-  </si>
-  <si>
-    <t>9fa304375ed23f8122c199f18ec0d5ce</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.54291d40c2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>17:56:07+00:00</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.69c250f5e6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>c341dff041650483e8e6d03b9cdadcd5</t>
-  </si>
-  <si>
-    <t>18:06:01+00:00</t>
-  </si>
-  <si>
     <t>subject_application_id: TELERICETTA</t>
   </si>
   <si>
@@ -2159,6 +2114,51 @@
   </si>
   <si>
     <t>L'errore viene trasmesso all'utente con il dettaglio del vocabolario non valido</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.223c4d535a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.b581d93d51^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>b9a2822074c8afeeefc9a42de66fb91f</t>
+  </si>
+  <si>
+    <t>210748a3431f15fc79645859adee2591</t>
+  </si>
+  <si>
+    <t>18:46:14+00:00</t>
+  </si>
+  <si>
+    <t>18:48:54+00:00</t>
+  </si>
+  <si>
+    <t>08:12:29+00:00</t>
+  </si>
+  <si>
+    <t>08:17:24+00:00</t>
+  </si>
+  <si>
+    <t>08:22:19+00:00</t>
+  </si>
+  <si>
+    <t>3c1a0552f25074505a4be623d57864a8</t>
+  </si>
+  <si>
+    <t>40d2f73b6847d2b652cacff9b5435eae</t>
+  </si>
+  <si>
+    <t>90f548f617d4dc6a411e78b6608aeede</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.c8dd407348^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.80d504f934^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.b706431650a2b3dc25e398723e8f20658fb17b6f990ace8f627b36e84474c6f4.68c493d044^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -2629,7 +2629,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2754,7 +2754,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2776,6 +2775,34 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4223,7 +4250,10 @@
     <col min="3" max="3" width="20.140625" customWidth="1"/>
     <col min="4" max="4" width="63.85546875" customWidth="1"/>
     <col min="5" max="5" width="104.85546875" customWidth="1"/>
-    <col min="6" max="9" width="33.140625" customWidth="1"/>
+    <col min="6" max="6" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="39.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="73.5703125" customWidth="1"/>
     <col min="10" max="10" width="27.140625" customWidth="1"/>
     <col min="11" max="18" width="36.42578125" customWidth="1"/>
     <col min="19" max="19" width="27.140625" customWidth="1"/>
@@ -4255,14 +4285,14 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="50"/>
-      <c r="C2" s="51" t="s">
-        <v>569</v>
-      </c>
-      <c r="D2" s="50"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="50" t="s">
+        <v>554</v>
+      </c>
+      <c r="D2" s="49"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -4283,14 +4313,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="53"/>
-      <c r="C3" s="58" t="s">
-        <v>566</v>
-      </c>
-      <c r="D3" s="50"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="57" t="s">
+        <v>551</v>
+      </c>
+      <c r="D3" s="49"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -4311,12 +4341,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="54"/>
-      <c r="B4" s="55"/>
-      <c r="C4" s="58" t="s">
-        <v>567</v>
-      </c>
-      <c r="D4" s="50"/>
+      <c r="A4" s="53"/>
+      <c r="B4" s="54"/>
+      <c r="C4" s="57" t="s">
+        <v>552</v>
+      </c>
+      <c r="D4" s="49"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -4338,12 +4368,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="56"/>
-      <c r="B5" s="57"/>
-      <c r="C5" s="58" t="s">
-        <v>568</v>
-      </c>
-      <c r="D5" s="50"/>
+      <c r="A5" s="55"/>
+      <c r="B5" s="56"/>
+      <c r="C5" s="57" t="s">
+        <v>553</v>
+      </c>
+      <c r="D5" s="49"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -4364,8 +4394,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="47"/>
-      <c r="B6" s="48"/>
+      <c r="A6" s="46"/>
+      <c r="B6" s="47"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -8994,64 +9024,64 @@
         <v>50</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="33">
+    <row r="129" spans="1:23" s="66" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="58">
         <v>168</v>
       </c>
-      <c r="B129" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="C129" s="39" t="s">
+      <c r="B129" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="C129" s="59" t="s">
         <v>57</v>
       </c>
-      <c r="D129" s="33" t="s">
+      <c r="D129" s="58" t="s">
         <v>272</v>
       </c>
-      <c r="E129" s="41" t="s">
+      <c r="E129" s="60" t="s">
         <v>273</v>
       </c>
-      <c r="F129" s="35">
-        <v>46096</v>
-      </c>
-      <c r="G129" s="35" t="s">
-        <v>552</v>
-      </c>
-      <c r="H129" s="45" t="s">
+      <c r="F129" s="61">
+        <v>46099</v>
+      </c>
+      <c r="G129" s="61" t="s">
+        <v>562</v>
+      </c>
+      <c r="H129" s="62" t="s">
+        <v>565</v>
+      </c>
+      <c r="I129" s="62" t="s">
+        <v>568</v>
+      </c>
+      <c r="J129" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="K129" s="63"/>
+      <c r="L129" s="63"/>
+      <c r="M129" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="N129" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="O129" s="62" t="s">
         <v>548</v>
       </c>
-      <c r="I129" s="45" t="s">
-        <v>549</v>
-      </c>
-      <c r="J129" s="36" t="s">
+      <c r="P129" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="K129" s="36"/>
-      <c r="L129" s="36"/>
-      <c r="M129" s="36" t="s">
+      <c r="Q129" s="63" t="s">
+        <v>543</v>
+      </c>
+      <c r="R129" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="N129" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="O129" s="45" t="s">
-        <v>550</v>
-      </c>
-      <c r="P129" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q129" s="36" t="s">
-        <v>543</v>
-      </c>
-      <c r="R129" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="S129" s="36" t="s">
-        <v>570</v>
-      </c>
-      <c r="T129" s="36"/>
-      <c r="U129" s="37"/>
-      <c r="V129" s="38"/>
-      <c r="W129" s="36" t="s">
+      <c r="S129" s="63" t="s">
+        <v>555</v>
+      </c>
+      <c r="T129" s="63"/>
+      <c r="U129" s="64"/>
+      <c r="V129" s="65"/>
+      <c r="W129" s="63" t="s">
         <v>50</v>
       </c>
     </row>
@@ -10336,16 +10366,16 @@
         <v>342</v>
       </c>
       <c r="F164" s="35">
-        <v>46096</v>
+        <v>46098</v>
       </c>
       <c r="G164" s="35" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="H164" s="35" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="I164" s="40" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="J164" s="36" t="s">
         <v>76</v>
@@ -10383,16 +10413,16 @@
         <v>344</v>
       </c>
       <c r="F165" s="35">
-        <v>46096</v>
+        <v>46098</v>
       </c>
       <c r="G165" s="35" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="H165" s="35" t="s">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="I165" s="45" t="s">
-        <v>563</v>
+        <v>557</v>
       </c>
       <c r="J165" s="36" t="s">
         <v>76</v>
@@ -10783,64 +10813,64 @@
         <v>47</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A176" s="33">
+    <row r="176" spans="1:23" s="66" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A176" s="58">
         <v>461</v>
       </c>
-      <c r="B176" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="C176" s="39" t="s">
+      <c r="B176" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="C176" s="59" t="s">
         <v>57</v>
       </c>
-      <c r="D176" s="33" t="s">
+      <c r="D176" s="58" t="s">
         <v>365</v>
       </c>
-      <c r="E176" s="41" t="s">
+      <c r="E176" s="60" t="s">
         <v>366</v>
       </c>
-      <c r="F176" s="46">
-        <v>46096</v>
-      </c>
-      <c r="G176" s="33" t="s">
-        <v>551</v>
-      </c>
-      <c r="H176" s="45" t="s">
-        <v>553</v>
-      </c>
-      <c r="I176" s="45" t="s">
-        <v>554</v>
-      </c>
-      <c r="J176" s="36" t="s">
+      <c r="F176" s="61">
+        <v>46099</v>
+      </c>
+      <c r="G176" s="58" t="s">
+        <v>563</v>
+      </c>
+      <c r="H176" s="62" t="s">
+        <v>566</v>
+      </c>
+      <c r="I176" s="62" t="s">
+        <v>569</v>
+      </c>
+      <c r="J176" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="K176" s="36"/>
-      <c r="L176" s="33"/>
-      <c r="M176" s="36" t="s">
+      <c r="K176" s="63"/>
+      <c r="L176" s="58"/>
+      <c r="M176" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="N176" s="36" t="s">
+      <c r="N176" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="O176" s="45" t="s">
+      <c r="O176" s="62" t="s">
+        <v>549</v>
+      </c>
+      <c r="P176" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q176" s="63" t="s">
+        <v>543</v>
+      </c>
+      <c r="R176" s="63" t="s">
+        <v>76</v>
+      </c>
+      <c r="S176" s="63" t="s">
         <v>555</v>
       </c>
-      <c r="P176" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q176" s="36" t="s">
-        <v>543</v>
-      </c>
-      <c r="R176" s="36" t="s">
-        <v>76</v>
-      </c>
-      <c r="S176" s="36" t="s">
-        <v>570</v>
-      </c>
-      <c r="T176" s="36"/>
-      <c r="U176" s="33"/>
-      <c r="V176" s="33"/>
-      <c r="W176" s="33" t="s">
+      <c r="T176" s="63"/>
+      <c r="U176" s="58"/>
+      <c r="V176" s="58"/>
+      <c r="W176" s="58" t="s">
         <v>50</v>
       </c>
     </row>
@@ -11329,64 +11359,64 @@
         <v>50</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A190" s="33">
+    <row r="190" spans="1:23" s="66" customFormat="1" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="58">
         <v>475</v>
       </c>
-      <c r="B190" s="33" t="s">
-        <v>43</v>
-      </c>
-      <c r="C190" s="39" t="s">
+      <c r="B190" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="C190" s="59" t="s">
         <v>57</v>
       </c>
-      <c r="D190" s="33" t="s">
+      <c r="D190" s="58" t="s">
         <v>393</v>
       </c>
-      <c r="E190" s="41" t="s">
+      <c r="E190" s="60" t="s">
         <v>394</v>
       </c>
-      <c r="F190" s="35">
-        <v>46096</v>
-      </c>
-      <c r="G190" s="35" t="s">
-        <v>559</v>
-      </c>
-      <c r="H190" s="35" t="s">
-        <v>556</v>
-      </c>
-      <c r="I190" s="40" t="s">
-        <v>557</v>
-      </c>
-      <c r="J190" s="36" t="s">
+      <c r="F190" s="61">
+        <v>46099</v>
+      </c>
+      <c r="G190" s="61" t="s">
+        <v>564</v>
+      </c>
+      <c r="H190" s="61" t="s">
+        <v>567</v>
+      </c>
+      <c r="I190" s="67" t="s">
+        <v>570</v>
+      </c>
+      <c r="J190" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="K190" s="36"/>
-      <c r="L190" s="36"/>
-      <c r="M190" s="36" t="s">
+      <c r="K190" s="63"/>
+      <c r="L190" s="63"/>
+      <c r="M190" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="N190" s="36" t="s">
+      <c r="N190" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="O190" s="45" t="s">
-        <v>558</v>
-      </c>
-      <c r="P190" s="36" t="s">
+      <c r="O190" s="62" t="s">
+        <v>550</v>
+      </c>
+      <c r="P190" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="Q190" s="36" t="s">
+      <c r="Q190" s="63" t="s">
         <v>543</v>
       </c>
-      <c r="R190" s="36" t="s">
+      <c r="R190" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="S190" s="36" t="s">
-        <v>570</v>
-      </c>
-      <c r="T190" s="36"/>
-      <c r="U190" s="37"/>
-      <c r="V190" s="38"/>
-      <c r="W190" s="36" t="s">
+      <c r="S190" s="63" t="s">
+        <v>555</v>
+      </c>
+      <c r="T190" s="63"/>
+      <c r="U190" s="64"/>
+      <c r="V190" s="65"/>
+      <c r="W190" s="63" t="s">
         <v>50</v>
       </c>
     </row>
@@ -16427,7 +16457,7 @@
   <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{F5F4AC7B-142E-4F14-AD0B-95E75DB6B433}">
           <x14:formula1>
             <xm:f>Sheet1!$B$2:$B$3</xm:f>
@@ -18736,6 +18766,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
+    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -18999,28 +19050,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a56712a3-8dfd-4688-917a-22f0cf513b89" xsi:nil="true"/>
-    <UserStoryALM xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1e76d14e-d0ce-457c-8343-9b55836d9ead">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19039,31 +19094,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C4C806F-EC4E-4231-9462-6D32094C4603}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="a56712a3-8dfd-4688-917a-22f0cf513b89"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{e0793d39-0939-496d-b129-198edd916feb}" enabled="0" method="" siteId="{e0793d39-0939-496d-b129-198edd916feb}" removed="1"/>

</xml_diff>